<commit_message>
se actualizo la portada de los destacados
</commit_message>
<xml_diff>
--- a/ofertas.xlsx
+++ b/ofertas.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
+  <dimension ref="A1:M104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="3" min="1" max="1"/>
@@ -1171,12 +1171,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cocinero (básico) turno mañana</t>
+          <t>Cocinero y ayudantes de cocina (PITT TIEN)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hotel Santa Isabel</t>
+          <t>PITT TIEN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Urgente busca personal responsable: cocinero (básico) para turno mañana. Sueldo a tratar. Referencia: Hotel Santa Isabel, Av. San Martín / Plazoleta Unidad Vecinal. Solo WhatsApp.</t>
+          <t>PITT TIEN está contratando: cocinero, ayudante de cocina con experiencia y ayudante de cocina con o sin experiencia. Sueldo justo, acuerdo al mercado y pagos puntuales. Ubicación: Av. San Martín, esquina Hotel Santa Isabel (Espinar). Comunicarse por llamada al 956102670 o por WhatsApp al 910006315.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Se necesitan 2 ayudantes de cocina (señora, señorita o joven) y 1 moza, tiempo completo, para restaurante en Espinar. Trato por llamada.</t>
+          <t>Se necesitan 2 ayudantes de cocina (señora, señorita o joven), en medio tiempo de 3:00 p.m. a 9:00 p.m. o en tiempo completo, y 1 moza en tiempo completo o medio tiempo, para restaurante en Espinar. Trato por llamada.</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2167,7 +2167,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -3637,13 +3637,11 @@
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>Sé parte de grandes retos y crece con nosotros en Antapaccay. Enviar CV a: 994 433 777 / 959 000 549. Beneficios: movilidad mensual. Construyendo juntos un futuro mejor.</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>994433777</t>
@@ -3684,19 +3682,16 @@
           <t>Vendedora y apoyo en tienda de cerámicas</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>Urgente: una señorita para ventas y un joven para apoyo en tienda de cerámicas. Dirección: Av. San Martín 507. CEL: 996 006 035 / 956 760 688.</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>996006035</t>
@@ -3737,19 +3732,16 @@
           <t>Maestro perforista (cobre) y 2 peones</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>Maestro perforista con experiencia/conocimiento en cobre y dos peones. Interesados dejar mensaje por WhatsApp o llamar, de 12:00pm a 1:30pm. CEL: 932 875 727.</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr">
         <is>
           <t>932875727</t>
@@ -3790,19 +3782,16 @@
           <t>Personal de limpieza para hotel</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>Hotel exclusivo requiere urgente una persona para limpieza, trabajo permanente. CEL: 959 745 906.</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>959745906</t>
@@ -3843,7 +3832,6 @@
           <t>Niñera para cuidar a dos niñas</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
@@ -3859,7 +3847,6 @@
           <t>Señorita responsable para cuidar dos niñas, se brinda alimentación, habitación y buen trato. Sueldo: S/1,700.00. CEL: 912 882 120.</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>912882120</t>
@@ -3900,7 +3887,6 @@
           <t>Jaladores para Espinar y Juliaca</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
@@ -3916,7 +3902,6 @@
           <t>Se necesita urgente jaladores. Pago quincenal S/1,000.00 y mensual S/2,000.00. Para Espinar y Juliaca. CEL: 912 882 120.</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
         <is>
           <t>912882120</t>
@@ -3957,7 +3942,6 @@
           <t>Atención al cliente en tienda de telecomunicaciones</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
@@ -3973,7 +3957,6 @@
           <t>Jóvenes y señoritas para atención al cliente en tienda de telecomunicaciones, c/s experiencia, con facilidad de palabras. Sueldo fijo S/1,500 más incentivos. CEL: 912 882 120.</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
           <t>912882120</t>
@@ -4014,7 +3997,6 @@
           <t>Cocinero(a) para El Descanso</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>El Descanso (40 min de Espinar) - Cusco</t>
@@ -4030,7 +4012,6 @@
           <t>Se necesita un cocinero(a) para 'El Descanso', a 40 min de Espinar. Se paga de S/2,500 a más. Interesados llamar al: CEL 915 229 427 / 953 286 230.</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr">
         <is>
           <t>915229427</t>
@@ -4071,19 +4052,16 @@
           <t>Personal de limpieza para hotel (medio tiempo) y ayudante de cocina</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>Urgente: personal de limpieza para hotel en medio tiempo y ayudante de cocina. CEL: 925 610 536 / 958 566 918.</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
           <t>925610536</t>
@@ -4124,19 +4102,16 @@
           <t>Atención en librería - internet (medio tiempo)</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>Joven o señorita para atención de librería - internet, medio tiempo, c/s experiencia. CEL: 956 604 147 / 930 384 715.</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr">
         <is>
           <t>956604147</t>
@@ -4177,19 +4152,16 @@
           <t>Atención al cliente en Agencia Shalom Encomiendas</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>Se requiere urgente jóvenes con experiencia y ganas de trabajar en atención al cliente. Interesados escribir al WhatsApp: 931 759 057.</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>931759057</t>
@@ -4230,19 +4202,16 @@
           <t>Conductores categoría A-IIC y A-IIB para transporte de personal</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>Conductores con categoría A-IIC y A-IIB, con experiencia de tres años, con brevete para transporte de personal. Enviar currículum al WhatsApp y/o llamar al: CEL 932 384 102.</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr">
         <is>
           <t>932384102</t>
@@ -4283,19 +4252,16 @@
           <t>Mozos(as) y ayudante de cocina</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>Restaurante en Cusco - Espinar requiere urgente mozos(as) c/s experiencia y ayudante de cocina. Requisitos: buena presencia, facilidad de palabra, ganas de trabajar. Horario 5:00pm-1:00am / 5:00pm-5:00am. Beneficios: alimentación (cena y desayuno), vivienda (opcional) o movilidad. Sistema 5 a 6 días laborados. Dirección: Plaza de Armas con Av. Arequipa. Llamadas: 984 329 666 / WhatsApp: 957 249 676.</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>957249676</t>
@@ -4336,19 +4302,16 @@
           <t>Mozas de línea y vajillero (concesionaria de alimentos)</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>Espinar - Cusco</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>Empresa concesionaria de alimentos requiere personal con experiencia en comedor: 02 mozas de línea y 01 vajillero. Horario con régimen minero 14x7, el trabajo es en Espinar. Beneficios: alimentación, hospedaje y movilidad. Enviar CV y/o comunicarse al WhatsApp: CEL 959 700 225 / 931 512 089.</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
           <t>959700225</t>
@@ -4377,6 +4340,1536 @@
       <c r="M74" t="inlineStr">
         <is>
           <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Ayudante de cocina, bajillero y mozos (concesionaria)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Para concesionaria se requiere: 1 ayudante de cocina con experiencia, 1 bajillero o bajillera (medio tiempo o tiempo completo) y 2 mozos o mozas (tiempo completo o medio tiempo). Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>940831074</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2 personas para carwash (contratación inmediata)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Se necesita contratación inmediata de 2 personas para trabajar en carwash, con disponibilidad inmediata, puntualidad y ganas de trabajar. Se ofrece buen ambiente laboral y pago competitivo a tratar. Los interesados deben comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>993155333</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>02 ayudantes para cargar, descargar y distribuir gas</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Se requiere de 02 ayudantes para cargar, descargar gas y distribuir. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>968590996</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Cocineros, cajeras, mozas y meseras para restaurante (apertura)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Con urgencia se necesita para restaurante en apertura: cocinero(a) con experiencia que sepa preparar ceviche y chicharrón de chancho, 02 cajeras, 03 mozas y 03 meseras de buena presencia. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>910188719</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Recepcionista para hotel (2:00 p.m. a 9:00 p.m.)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita proactiva y responsable para atención en recepción de hotel, en el horario de 2:00 p.m. a 9:00 p.m.</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>958152303</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Moza o ayudante para Pizzas de Freddy (2:40 p.m. a 11:00 p.m.)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Pizzas de Freddy necesita 02 personas (señorita o señora) o joven para moza o ayudante, en el horario de 2:40 p.m. a 11:00 p.m.</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>975215425</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Asistente contable, asistente de administración y oficios de construcción</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Se necesita: asistente contable, asistente de administración, soldadores, mecánicos, carpinteros y encofradores. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>938289220</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Vajillera</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita o señora para vajillera. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>957781614</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Técnica en farmacia o enfermería para botica</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Se requiere señorita técnica en farmacia o en enfermería para Espinar, para laborar en botica, con disponibilidad inmediata.</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>940879960</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Jóvenes para delivery</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Se necesitan jóvenes para delivery, con disponibilidad inmediata. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>949703993</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Señora o señorita para limpieza en hospedaje</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Con mucha urgencia se necesita una señora o señorita para trabajo en limpieza en un hospedaje. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>974277627</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Señorita de buena presencia, tiempo completo o medio tiempo</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>S/ 1,600</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Se necesita señorita de buena presencia, con o sin experiencia, de tiempo completo o medio tiempo. Remuneración S/ 1,600.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>966179195</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>02 personal para limpieza de hospedaje y persona responsable</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Se necesita 02 personal para limpieza de hospedaje (medio tiempo) y una persona responsable con trabajo fijo. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>956760688</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Señora o señorita para cuidado de 3 niños</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Arequipa</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Se necesita señora o señorita para cuidado de 3 niños en Arequipa, con facilidad de estudios y trato familiar. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>972930114</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Ayudante de cocina y mozo</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Se requiere un ayudante de cocina y mozo para Espinar, con disponibilidad inmediata y trato familiar. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>974410495</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Señorita para limpieza de hospedaje</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Se necesita señorita para limpieza de hospedaje. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>910916143</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Personal para hotel (referencia terminal antiguo)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Se necesita personal para hotel, con referencia en el terminal antiguo. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>959164789</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1 pollero y 1 cocinero para Santo Tomás</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Santo Tomás - Cusco</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Se necesita un pollero y un cocinero para Santo Tomás. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>900080146</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Señora o señorita para limpieza de hospedaje (2)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Se necesita una señora o señorita para limpieza de hospedaje. Llamar al número indicado.</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>958769976</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Señorita con conocimiento en cosmetología</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita que tenga conocimiento en cosmetología. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>964365593</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Urgente: ayudante para camión</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Urgente se necesita un ayudante para camión. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>998474614</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1 pollero y 1 cocinero para Santo Tomás (otro número)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Santo Tomás - Cusco</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Se necesita un pollero y un cocinero para Santo Tomás. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>967195137</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Técnica en farmacia o enfermería (se aceptan practicantes)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Se necesita técnica en farmacia o enfermería con experiencia, tiempo completo o medio tiempo. También se aceptan practicantes. Dirección: Av. Sol, Espinar.</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>969330822</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Señorita para restobar</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita para restobar. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>984792226</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Ayudante mecánico automotriz</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Se necesita ayudante mecánico automotriz. Comunicarse por llamada.</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>957061565</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Operador de cargador frontal</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Maquinaria y Servicios Alto Huarca S.A.</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Estamos en la búsqueda del mejor talento para unirse a nuestras operaciones en Espinar, Cusco, con experiencia en minería y con los estándares de seguridad de Antapaccay. Requisitos: formación de Técnico en Operación de Maquinaria Pesada (certificado); mínimo 3 años de experiencia en operación de cargador frontal en minería; conocimientos de normas de seguridad y mantenimiento básico de equipos; trabajo en equipo y responsabilidad. Régimen 14x7, salario acorde a experiencia.</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>959319697</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Operador de tractor oruga</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Maquinaria y Servicios Alto Huarca S.A.</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Estamos en la búsqueda del mejor talento para unirse a nuestras operaciones en Espinar, Cusco, con experiencia en minería y con los estándares de seguridad de Antapaccay. Requisitos: formación de Técnico en Operación de Maquinaria Pesada (certificado); mínimo 3 años de experiencia en operación de tractor oruga en minería; conocimientos de normas de seguridad y mantenimiento básico de equipos; trabajo en equipo y responsabilidad. Régimen 14x7, salario acorde a experiencia.</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>959319697</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Operador de excavadora</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Maquinaria y Servicios Alto Huarca S.A.</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Estamos en la búsqueda del mejor talento para unirse a nuestras operaciones en Espinar, Cusco, con experiencia en minería y con los estándares de seguridad de Antapaccay. Requisitos: formación de Técnico en Operación de Maquinaria Pesada (certificado); mínimo 3 años de experiencia en operación de excavadora en minería; conocimientos de normas de seguridad y mantenimiento básico de equipos; trabajo en equipo y responsabilidad. Régimen 14x7, salario acorde a experiencia.</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>959319697</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Atención al cliente, logística, distribución y empaquetado</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>S/ 1,250 + almuerzo</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Se requieren personales de 18 a 25 años con experiencia para atención al cliente, logística, distribución y empaquetado. Ingreso S/ 1,250 más almuerzo.</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>917799231</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Técnico de planos (construcción civil o cadista)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Consultora y Constructora Edifica</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Consultora y Constructora Edifica requiere un profesional: egresado, bachiller técnico o titulado por un instituto de diferentes especialidades, con educación superior tecnológico en construcción civil o cadista. Funciones: dibujo técnico de planos de diferentes especialidades, lectura e interpretación de planos, apoyo en el control de avance de planos de obra y apoyo en el desarrollo de proyectos de vivienda. Ofrecemos: grato ambiente laboral, oportunidad de crecimiento profesional, capacitación constante y participación en proyectos reales de arquitectura y construcción. Contacto: 949302068 / 918154152.</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>949302068</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>llamada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se suben las fotos del 21/10: 51 ofertas nuevas en ofertas.xlsx
</commit_message>
<xml_diff>
--- a/ofertas.xlsx
+++ b/ofertas.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M104"/>
+  <dimension ref="A1:M155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="3" min="1" max="1"/>
@@ -5873,6 +5873,2631 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Señorita para limpieza de hotel (Tintaya - Marquiri)</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Tintaya - Cusco</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita para limpieza de hotel en Tintaya - Marquiri.</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>900597981</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Mecánico automotriz con experiencia</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Se necesita mecánico automotriz con experiencia. Ingreso a planilla con todos los beneficios de ley y sueldo acorde al mercado.</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>957061565</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Señorita para moza y señorita o joven para valillería</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Se necesita urgente: señorita para moza y señorita o joven para valillería. Se paga buen sueldo y buen trato. Solo para Espinar.</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>983361223</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Señorita para cuidado de niña de 3 años</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita con experiencia para cuidado de una niña de 3 años, solo por días. Trato familiar.</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>978644321</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>02 mozos(as) y 02 ayudantes de cocina</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Se necesita 02 mozos(as) y 02 ayudantes de cocina. También se comunica al 926 842 123.</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>978664185</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Operarios y oficiales civiles y mecánicos (parada de planta - servicios)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Metales S.R.L.</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Metales S.R.L. - PARADA DE PLANTA - SERVICIOS. Estamos en la búsqueda de tu talento: operario civil, operario mecánicos, oficial civil, oficial mecánicos, ayudantes y supervisor de seguridad. Requisitos generales: titular de Degrees y/o colegiado en Ingeniería según los requisitos del puesto; experiencia mínima de 3 años en minería desempeñándose como supervisor de seguridad; habilitado para CM Antapaccay (deseable); residir en Espinar, Cusco, Arequipa o Puno; residir en la ciudad de Espinar. De cumplir con los requisitos, enviar su CV actualizado y documentado al WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>974660842</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Personal para limpieza de hotel (Hotel Yaureñita)</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Se necesita personal de 20 años a más para limpieza de hotel (sea joven, señorita o pareja). Apersonarse al Hotel Yaureñita, Av. Sol al costado del antiguo terminal, o llamar al número.</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>930684864</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Señorita para cuidado de niño de 2 años y medio</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita para el cuidado de un niño de 2 años y medio, de 2:00 p.m. a 6:00 p.m.</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>942724044</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Pastor para fundo ganadero</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>S/ 1,500</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Se busca pastor para fundo ganadero San Sebastián, en Alto Pichigua, sector Ccahuaya Alta, Espinar. Se necesita persona responsable para el cuidado del ganado en el fundo. Inicio inmediato. Se ofrece sueldo de S/ 1,500, vivienda incluida, trabajo estable y buen trato. Se acepta persona sola o pareja.</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>952827582</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Vajillero(a) para concesionaria de alimentos</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Se necesita vajillero(a) para concesionaria de alimentos, con régimen 20x10 e ingreso a planilla.</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>927584950</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Conductores de omnibus y camioneta para mina Las Bambas</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Challhuahuacho - Apurimac</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Empresa dedicada al transporte de personal en la mina Las Bambas - Challhuahuacho. Se busca conductores de omnibus y camioneta, con licencia de conducir A-IIB y A-IIC. Interesados enviar su CV al WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>997147179</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Pollero para pollería</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Pollería - estamos buscando pollero. Requisitos: experiencia comprobable (excluyente), saber trozar y filetear, conocimiento en elaboración de especialidades, ser rápido y tener ganas de trabajar, varón mayor de 18 años. Ofrecemos buen pago, negocio familiar y chico. Comunicarse al WhatsApp 958 738 195 / 983 150 367.</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>958738195</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Asesor(a) de ventas</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Operaciones Minero Metalúrgico S.A.C.</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Operaciones Minero Metalúrgico S.A.C. - Únete a nuestro equipo y crece con nosotros. Requisitos: experiencia mínima de 6 meses en ventas de productos industriales; habilidades de comunicación y negociación; actitud proactiva, responsable y orientada a resultados; manejo de WhatsApp Business, redes sociales y Excel básico; disponibilidad para trabajo presencial o de campo. Te ofrecemos: sueldo fijo más comisiones atractivas, capacitación constante y línea de carrera, buen ambiente laboral y respaldo de la empresa, todos los beneficios de ley.</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>916022558</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Personal para Antapaccay (supervisor HSE, topógrafo, operarios y oficiales civiles, operario electricista, conductor múltiple)</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Grupo Pedrisa</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Antapaccay - Cusco</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>PEDRISA (Grupo Pedrisa) - se requiere personal para Antapaccay: supervisor HSE, topógrafo, operarios civiles, oficiales civiles, ayudantes civiles, operario electricista y conductor múltiple. Requisitos: licencia interna activa y pase vigente para Antapaccay. Zona Sur, Calle Anta, Espinar - Cusco.</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>968787641</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Personal para Antapaccay (almacenero de mina, operarios y oficiales civiles, conductores, rigger, soldadores y mecánicos)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Grupo Pedrisa</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Antapaccay - Cusco</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>PEDRISA (Grupo Pedrisa) - se requiere: almacenero de mina, operarios civiles, oficiales civiles, ayudantes civiles, conductor de minibús, conductor de camión baranda, rigger, soldadores y mecánicos. Requisitos: licencia interna activa y pase vigente para Antapaccay. Enviar CV documentado al correo empleos@grupopedrisa.com. Zona Sur, Calle Anta, Espinar - Cusco.</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>968787641</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Practicantes mecánicos y mecánicos (Autrisa)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Autrisa</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>AUTRISA nos encontramos en la búsqueda de practicantes mecánicos y mecánicos nivel 1. Requisitos: egresado de mecánica automotriz, mantenimiento de maquinaria pesada o afines; conocimientos en mantenimiento preventivo y correctivo en unidades pesadas (VOLVO); disponibilidad para laborar en Espinar, carretera Espinar - Tintaya km 1.5, pasando puente de la amistad. Pago en planilla con todos los beneficios de ley. Envía tu CV al 973 588 457 / 980 608 243.</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>973588457</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Operadores y mecánicos para mina San Cristóbal (Caylloma - Arequipa)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Cristobal</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Caylloma - Arequipa</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>BATEAS - UM San Cristóbal (Caylloma, Arequipa). Se requiere: operadores jumbo múltiple, operadores bolter, operadores scaler, operador de scoop, ayudantes cargadores, mecánicos trackless M1-M2, operadores de volquete, mecánicos de volquete y conductores múltiple. Sistema 14x7, bonos, planilla desde el primer día, alimentación y vivienda cubierta 100% (Juliaca, Espinar y Arequipa), gratificación, CTS, asignación familiar, vacaciones, EsSalud y movilidad. Comunicarse por WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>988657086</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Mecánicos y montajistas para proyectos mineros</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>INIDEC</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>INIDEC - calidad en proyectos mineros. Se requiere mecánicos y montajistas. Ingreso a planilla y beneficios de ley. Habilitados para Antapaccay y habilitados para el 15 de octubre. Espinar - Cusco. Comunicarse al 910 514 777 / 931 880 188.</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>910514777</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Conductor de cisterna y furgón de succión de baños (Proyecto Antapaccay)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Antapaccay</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>S/ 1,900</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Proyecto Antapaccay - se busca conductor de cisterna / furgón de succión de baños. Requisitos: licencia de conducir A2B o A3C vigente, mínimo 3 años de experiencia comprobada como conductor, experiencia certificada con certificados de trabajo, disponibilidad para trabajar bajo régimen 14x7. Ofrecemos: S/ 1,900 en planilla completa (pago mensual), todos los beneficios de ley al 100%, gratificaciones al 100%, CTS al 100%, 30 días de vacaciones, alimentación cubierta y movilidad cubierta. Te recogemos desde Espinar y te trasladamos a Marquiri, con retorno al finalizar la jornada. Envía tu CV al 959 000 549 / 994 433 777.</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>959000549</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Señora de limpieza para hospedaje (medio tiempo)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Trabajo en hospedaje. Se necesita señora de limpieza, medio tiempo de 8:00 a.m. a 1:00 p.m., con experiencia.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>974359134</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Ayudante para campo Huisa Ccollana</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Urgente se necesita un joven o cualquier persona para ayudante en el campo Huisa Ccollana. Solo para ayudar a cercar ganado y cambiar y dar forraje. También se comunica al 974 388 692.</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>985737327</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Señoritas para venta de ropa</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Urgente se necesita señoritas para venta de ropa, con experiencia, turno tarde y mañana.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>972930114</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Ayudante de cocina para comedor universitario</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Se necesita 01 ayudante de cocina para el comedor universitario de Espinar.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>976188945</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Señoritas para juguería, desayunos, moza y ayudante de cocina</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Se necesita: 01 señorita para juguería turno mañana, 02 señoritas para desayunos turno mañana, 01 moza turno tarde y 01 ayudante de cocina.</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>944557348</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Mozos(as), vajillero y ayudante de cocina</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Se necesita: mozos(as), vajillero y ayudante de cocina.</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>959867892</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>01 mozo(a) y 01 ayudante de cocina</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Se necesita 01 mozo(a) y 01 ayudante de cocina. También se comunica al 926 842 123.</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>978664185</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Señorita o joven para atención al cliente en restaurante</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Se necesita señorita o joven para atención al cliente para un restaurante.</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>959867892</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Moza y lavavajilla para restaurante</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Urgente se necesita 01 moza y 01 lavavajilla, de 8:00 a.m. a 4:00 p.m., para un restaurante.</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>919685662</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Señora o caballero para ayudante de cocina y señorita o joven para atención al cliente</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Se necesita señora o caballero para ayudante de cocina y señorita o joven para atención al cliente.</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>959867892</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Señorita para moza (Cama Adentro)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita para moza para el distrito de Cama Adentro. Trato familiar. También se comunica al 991 601 037.</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>950233483</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Moza y ayudante general para concesionaria de alimentos</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Se requiere personal para concesionaria de alimentos: 1 moza turno tarde de 3:00 p.m. a 8:30 p.m. y 1 ayudante general. Lugar de trabajo: Espinar, Cusco.</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>989574246</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Asistente de apoyo para dibujo de planos y atención de oficina</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Oportunidad de trabajo: se requiere un asistente de apoyo para dibujo de planos y atención de oficina.</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>900131626</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Vajillero para Caylloma</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Caylloma - Arequipa</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>S/ 2,000</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Urgente se necesita un vajillero, sueldo 2,000 soles, con experiencia, para Caylloma.</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>983877353</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Atención de cabina de internet</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Se necesita personal para atención de cabina de internet: un joven (sin experiencia) con disponibilidad inmediata de 7:00 p.m. a 12:00 a.m. de lunes a domingo. También se comunica al 921 033 430.</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>997173817</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Niñera responsable para cuidar 2 niñas</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Se busca una niñera responsable para cuidar 2 niñas, de preferencia de 20 a 30 años. Lugar de trabajo: Espinar. Buen sueldo y con sistema 14x7.</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>965396957</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Maestro perforista y 4 personales para minería</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Urgente se requiere 04 personales y 01 maestro perforista con experiencia para la minería. Se paga buen sueldo. También se comunica al 985 989 816.</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>948265262</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Personal para restaurante Machupicchu</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Machupicchu - Cusco</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Restaurante Machupicchu se requiere personal: cocinero, ayudante de cocinera, mozos(as), vajilleros y limpieza. Todos con experiencia.</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>949745375</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Señorita o voluntario(a) para seguridad en barra y eventos (Apolo's Disco Club)</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Apolo's Disco Club</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Únete a nuestro equipo. Se necesita señorita o voluntario(a) de buena presencia para seguridad en barra y eventos, con responsabilidad. Comunicarse al 946 995 424. Dirección: Alfonso Ugarte 310, a 2 cuadras de la Plaza de Armas, Espinar - Cusco.</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>946995424</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Psicólogo(a) y técnico en seguridad y salud en el trabajo</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Apu Llallawa</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Apu Llallawa - Únete a nuestra gran familia. 1) Titulado, colegiado y habilitado en Psicología; acreditar experiencia en cargos similares, mínimo de 1 año; liderazgo y compromiso; comunicación efectiva y trabajo en equipo; capacidad de gestión de personas; conocimiento de conceptos de seguridad y salud; disponibilidad para trabajar en Espinar, bajo régimen atípico 2x1. 2) Técnicos y/o universitarios de ingeniería de seguridad, ambiental, industrial, computación y/o carreras afines; experiencia certificada de más de 1 año en el puesto; residir en la zona sur del Perú; disponibilidad para trabajar bajo régimen de 9x6. También se comunica al 986 762 345.</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>932558281</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Señorita para apoyo en restaurante</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Se necesita señorita para apoyo en restaurante, de lunes a viernes medio tiempo, sábado y domingo tiempo completo.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>959565714</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Moza y atención al cliente (Patronal Restobar)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Patronal Restobar</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Patronal Restobar - trabaja con nosotros. Puesto: moza y atención al cliente. Lugar: Espinar. Horario: tarde y noche. Ofrecemos sueldo excelente, bonos, capacitación pagada, buen ambiente y respeto. Escribe al WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>950122218</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Personal para incorporarse al equipo de trabajo</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>¿Quieres aprender un oficio dinámico y con futuro? ¡Esta es tu oportunidad! Estamos incorporando personas responsables a nuestro equipo de trabajo. Requisitos: tener ganas de trabajar y aprender.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>935437854</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Ingeniero de seguridad (Antapaccay - Espinar)</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Se requiere ingeniero de seguridad: experiencia mínima de 3 años en seguridad, con experiencia en trabajos de soldadura y mantenimiento industrial. Antapaccay - Espinar. Sistema 14x14. Interesados enviar CV por interno. También se comunica al 958 701 609.</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>967408092</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Señorita para atención al cliente y ventas</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>S/ 2,000</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita con o sin experiencia en atención al cliente para ventas. Remuneración de S/ 2,000 mensual.</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>951753064</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Moza y ayudante de cocina</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Se necesita urgente: 1 moza y 1 ayudante de cocina.</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>974782159</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Señorita para tienda de ferretería</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Se solicita una señorita responsable, puntual y con ganas de aprender, con o sin experiencia, para una tienda de ferretería.</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>984719613</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Señorita para tienda comercial Pichiguianito</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Se necesita una señorita para trabajar en la tienda comercial Pichiguianito. Horarios: jueves y viernes de 3:00 p.m. a 8:00 p.m.; sábados y domingos de 8:00 a.m. a 8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>989487038</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Ayudante de cocina para establecimiento en Marquiri</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Tintaya - Cusco</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>¡Contratando! Buscamos personal responsable, dinámico y con ganas de trabajar para nuestro establecimiento en Marquiri: 1 ayudante de cocina. Ofrecemos buen ambiente de trabajo, respeto, compromiso y oportunidad de crecimiento.</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>930761491</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Personal de construcción para subestación (Tintaya)</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Tintaya - Cusco</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Construcción para la subestación Tintaya, régimen civil. Se requiere: oficiales carpinteros, operario albañil, operario fierrero, operario carpintero y oficial de instalación eléctrica. Ofrecemos buen ambiente laboral, estabilidad en el trabajo y proyecto de gran importancia. También se comunica al 944 088 488.</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>914905717</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Técnica en farmacia o enfermería</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Se necesita técnica en farmacia o enfermería, con experiencia, tiempo completo.</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>925528020</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Cocinero(a), cajera y tres mozas para restobar</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Espinar - Cusco</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Se necesita con urgencia para restobar: cocinero(a) que sepa preparar ceviche y chicharrón de chancho, cajera y tres mozas de buena presencia.</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>910188719</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>llamada</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Se agrega la oferta de QORITICLLA S.A.C. (WA0066) y se corrigen tildes
</commit_message>
<xml_diff>
--- a/ofertas.xlsx
+++ b/ofertas.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:M156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="3" min="1" max="1"/>
@@ -8498,6 +8498,61 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Operarios, oficiales, peones y operadores de retroexcavadora (obra de torres de alta tensión)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>QORITICLLA S.A.C</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Chocñihuaqui - Arequipa</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>¡Únete a nuestro equipo de trabajo! OBRA: construcción de obras de cimentación para torres de alta tensión. LUGAR DE TRABAJO: Comunidad de Chocñihuaqui, distrito de Cayarani, provincia de Condesuyos, departamento de Arequipa. PERSONAL REQUERIDO: 10 operarios (múltiples), 10 oficiales (múltiples), peones y operadores de retroexcavadora. Régimen 20x10. Los interesados pueden enviar su CV al correo qoriticlla.gerencia@gmail.com o al número de WhatsApp.</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>997601198</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>